<commit_message>
fix export and message
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ExportOrderTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ExportOrderTemplate.xlsx
@@ -81,33 +81,34 @@
       <family val="0"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <b val="true"/>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF9FC5E8"/>
-        <bgColor rgb="FFC0C0C0"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -136,17 +137,13 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -158,66 +155,6 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF9FC5E8"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -226,15 +163,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr defaultColWidth="12.640625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr defaultColWidth="12.66015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="23.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="6.39"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -256,13 +194,14 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
update 2 template export excel file
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ExportOrderTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ExportOrderTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\working\source\23-kcvn-spm-be\src\main\kotlin\com\kcvn\spm\assets\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\working\source\23-kcvn-spm-be\target\classes\assets\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{102D49C5-CF2D-488C-A727-E53DE56A59A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{533D73E2-CD6F-4DF0-B6EC-423483023235}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="38700" windowHeight="15345" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Đơn Hàng" sheetId="1" r:id="rId1"/>

</xml_diff>